<commit_message>
remove osm cache to ra2ce
</commit_message>
<xml_diff>
--- a/work_dir/output/hazard_names.xlsx
+++ b/work_dir/output/hazard_names.xlsx
@@ -453,7 +453,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>hazard</t>
+          <t>hazard_new_crs</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -468,14 +468,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>C:\Users\hauth\repositories\ra2ce-viktor\work_dir\static\hazard\hazard.tif</t>
+          <t>C:\Users\hauth\repositories\ra2ce-viktor\work_dir\static\hazard\hazard_new_crs.tif</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>hazard</t>
+          <t>hazard_new_crs</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>C:\Users\hauth\repositories\ra2ce-viktor\work_dir\static\hazard\hazard.tif</t>
+          <t>C:\Users\hauth\repositories\ra2ce-viktor\work_dir\static\hazard\hazard_new_crs.tif</t>
         </is>
       </c>
     </row>

</xml_diff>